<commit_message>
Add document extraction script; fix malformed source URLs
extract_documents.py downloads government documents listed in the research
spreadsheet into category-organized folders, with self-describing filenames
(source slug + original name + URL hash to guarantee uniqueness even when
a site serves distinct documents through a generic query-string path).
Handles multi-URL cells, relative-path shorthand, TLS-cert-broken sites
(--insecure-tls), and writes a full provenance manifest per file.

Also corrects two malformed Document URL entries found while testing: a
truncated Bihar link and a Telangana row with prose embedded in the URL
cell.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/india_traffic_document_links.xlsx
+++ b/research/india_traffic_document_links.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Document Source Links'!$A$1:$F$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Document Source Links'!$A$1:$F$127</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -659,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F126"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1947,7 +1947,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>https://state.bihar.gov.in/transport/SectionInformation.html?editForm&amp;rowId=964 | rowId=4065</t>
+          <t>https://state.bihar.gov.in/transport/SectionInformation.html?editForm&amp;rowId=964 | https://state.bihar.gov.in/transport/SectionInformation.html?editForm&amp;rowId=4065</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -4041,7 +4041,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Siddipet / Nizamabad Districts (Telangana) - Road Safety Committee Minutes</t>
+          <t>Siddipet District (Telangana) - Road Safety Committee Minutes</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>https://siddipet.telangana.gov.in/ | https://nizamabad.telangana.gov.in/ (path: /minutes-of-...-road-safety-committee-meetings/)</t>
+          <t>https://siddipet.telangana.gov.in/minutes-of-district-road-safety-committee-meetings/</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -4064,12 +4064,16 @@
           <t>Search-result only</t>
         </is>
       </c>
-      <c r="F111" s="4" t="inlineStr"/>
+      <c r="F111" s="4" t="inlineStr">
+        <is>
+          <t>Path pattern per source agent report; exact slug not independently confirmed</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>North East District (Delhi) - District Road Safety Committee</t>
+          <t>Nizamabad District (Telangana) - Road Safety Committee Minutes</t>
         </is>
       </c>
       <c r="B112" s="16" t="inlineStr">
@@ -4079,7 +4083,7 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>https://dmnortheast.delhi.gov.in/district-road-safety-committee/</t>
+          <t>https://nizamabad.telangana.gov.in/minutes-of-district-road-safety-committee-meetings/</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -4092,12 +4096,16 @@
           <t>Search-result only</t>
         </is>
       </c>
-      <c r="F112" s="4" t="inlineStr"/>
+      <c r="F112" s="4" t="inlineStr">
+        <is>
+          <t>Path pattern per source agent report; exact slug not independently confirmed</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Chandigarh Transport Undertaking - DLRSC Minutes</t>
+          <t>North East District (Delhi) - District Road Safety Committee</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
@@ -4107,12 +4115,12 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>https://chdctu.gov.in/minutes-of-meetings-of-district-road-safety-committee-dlrsc</t>
+          <t>https://dmnortheast.delhi.gov.in/district-road-safety-committee/</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>District/UT-level Road Safety Committee minutes</t>
+          <t>DRSC minutes</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -4125,7 +4133,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Patna District (Bihar) - DM Orders</t>
+          <t>Chandigarh Transport Undertaking - DLRSC Minutes</t>
         </is>
       </c>
       <c r="B114" s="16" t="inlineStr">
@@ -4135,29 +4143,25 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>https://patna.nic.in/notice/district-magistrate-order-patna/ | /district-magistrate-office-order-patna/</t>
+          <t>https://chdctu.gov.in/minutes-of-meetings-of-district-road-safety-committee-dlrsc</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>District Magistrate orders</t>
-        </is>
-      </c>
-      <c r="E114" s="6" t="inlineStr">
-        <is>
-          <t>Partial / Unconfirmed</t>
-        </is>
-      </c>
-      <c r="F114" s="4" t="inlineStr">
-        <is>
-          <t>SSL certificate expired on both http/https attempts - needs re-verification</t>
-        </is>
-      </c>
+          <t>District/UT-level Road Safety Committee minutes</t>
+        </is>
+      </c>
+      <c r="E114" s="8" t="inlineStr">
+        <is>
+          <t>Search-result only</t>
+        </is>
+      </c>
+      <c r="F114" s="4" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>[PATTERN] District NIC template - Diversion Orders</t>
+          <t>Patna District (Bihar) - DM Orders</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
@@ -4167,29 +4171,29 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>https://&lt;district&gt;.nic.in/en/notice/diversion-order/</t>
+          <t>https://patna.nic.in/notice/district-magistrate-order-patna/ | /district-magistrate-office-order-patna/</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>Traffic diversion/prohibitory orders</t>
-        </is>
-      </c>
-      <c r="E115" s="8" t="inlineStr">
-        <is>
-          <t>Search-result only</t>
+          <t>District Magistrate orders</t>
+        </is>
+      </c>
+      <c r="E115" s="6" t="inlineStr">
+        <is>
+          <t>Partial / Unconfirmed</t>
         </is>
       </c>
       <c r="F115" s="4" t="inlineStr">
         <is>
-          <t>Scalable pattern confirmed across HP, MP, TN districts - apply across India's ~750 districts for systematic discovery</t>
+          <t>SSL certificate expired on both http/https attempts - needs re-verification</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>[PATTERN] District NIC template - Road Safety Committee Minutes</t>
+          <t>[PATTERN] District NIC template - Diversion Orders</t>
         </is>
       </c>
       <c r="B116" s="16" t="inlineStr">
@@ -4199,12 +4203,12 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>https://&lt;district&gt;.nic.in/document-category/minutes-of-meeting-of-district-road-safety-committee/</t>
+          <t>https://&lt;district&gt;.nic.in/en/notice/diversion-order/</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>District Road Safety Committee (DM/Collector-chaired) minutes</t>
+          <t>Traffic diversion/prohibitory orders</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
@@ -4214,46 +4218,46 @@
       </c>
       <c r="F116" s="4" t="inlineStr">
         <is>
-          <t>Scalable pattern confirmed across HP, MP (Almora), TN, Karnataka, Telangana, Delhi, Chandigarh</t>
+          <t>Scalable pattern confirmed across HP, MP, TN districts - apply across India's ~750 districts for systematic discovery</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>e-Courts - Motor Accident Claims Tribunal (MACT) district network</t>
-        </is>
-      </c>
-      <c r="B117" s="17" t="inlineStr">
-        <is>
-          <t>Judicial</t>
+          <t>[PATTERN] District NIC template - Road Safety Committee Minutes</t>
+        </is>
+      </c>
+      <c r="B117" s="16" t="inlineStr">
+        <is>
+          <t>District</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>https://districts.ecourts.gov.in/motor-accident-claims-tribunal</t>
+          <t>https://&lt;district&gt;.nic.in/document-category/minutes-of-meeting-of-district-road-safety-committee/</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>Index linking every district's MACT (rules, notifications, circulars, statistical reports)</t>
-        </is>
-      </c>
-      <c r="E117" s="5" t="inlineStr">
-        <is>
-          <t>Verified - Live</t>
+          <t>District Road Safety Committee (DM/Collector-chaired) minutes</t>
+        </is>
+      </c>
+      <c r="E117" s="8" t="inlineStr">
+        <is>
+          <t>Search-result only</t>
         </is>
       </c>
       <c r="F117" s="4" t="inlineStr">
         <is>
-          <t>Confirmed real document categories at sample district (mumact.dcourts.gov.in/documents/)</t>
+          <t>Scalable pattern confirmed across HP, MP (Almora), TN, Karnataka, Telangana, Delhi, Chandigarh</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Supreme Court Committee on Road Safety - Directions (HP mirror)</t>
+          <t>e-Courts - Motor Accident Claims Tribunal (MACT) district network</t>
         </is>
       </c>
       <c r="B118" s="17" t="inlineStr">
@@ -4263,29 +4267,29 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>https://roadsafety.hp.gov.in/storage/files/supreme%20court%20committee/Directions/</t>
+          <t>https://districts.ecourts.gov.in/motor-accident-claims-tribunal</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>Numbered sequence of binding SC committee directions to states on road safety</t>
-        </is>
-      </c>
-      <c r="E118" s="6" t="inlineStr">
-        <is>
-          <t>Partial / Unconfirmed</t>
+          <t>Index linking every district's MACT (rules, notifications, circulars, statistical reports)</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>Verified - Live</t>
         </is>
       </c>
       <c r="F118" s="4" t="inlineStr">
         <is>
-          <t>No single central SCCoRS website exists; directions are mirrored piecemeal on state portals - this HP directory looks systematically crawlable</t>
+          <t>Confirmed real document categories at sample district (mumact.dcourts.gov.in/documents/)</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Supreme Court - 'In Re: Highway Safety' suo-motu judgment (2026)</t>
+          <t>Supreme Court Committee on Road Safety - Directions (HP mirror)</t>
         </is>
       </c>
       <c r="B119" s="17" t="inlineStr">
@@ -4295,61 +4299,61 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>https://api.sci.gov.in/supremecourt/2025/63765/63765_2025_3_42_70046_Judgement_13-Apr-2026.pdf</t>
+          <t>https://roadsafety.hp.gov.in/storage/files/supreme%20court%20committee/Directions/</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>Full judgment: nationwide interim road-safety directions, District Highway Safety Task Forces, blackspot rectification</t>
-        </is>
-      </c>
-      <c r="E119" s="8" t="inlineStr">
-        <is>
-          <t>Search-result only</t>
+          <t>Numbered sequence of binding SC committee directions to states on road safety</t>
+        </is>
+      </c>
+      <c r="E119" s="6" t="inlineStr">
+        <is>
+          <t>Partial / Unconfirmed</t>
         </is>
       </c>
       <c r="F119" s="4" t="inlineStr">
         <is>
-          <t>Hosted on Supreme Court's own official API domain - very high-confidence primary legal source</t>
+          <t>No single central SCCoRS website exists; directions are mirrored piecemeal on state portals - this HP directory looks systematically crawlable</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>data.gov.in - Road Accidents dataset group</t>
-        </is>
-      </c>
-      <c r="B120" s="18" t="inlineStr">
-        <is>
-          <t>Research/Data/Statistics</t>
+          <t>Supreme Court - 'In Re: Highway Safety' suo-motu judgment (2026)</t>
+        </is>
+      </c>
+      <c r="B120" s="17" t="inlineStr">
+        <is>
+          <t>Judicial</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>https://www.data.gov.in/dataset-group-name/Road%20Accidents</t>
+          <t>https://api.sci.gov.in/supremecourt/2025/63765/63765_2025_3_42_70046_Judgement_13-Apr-2026.pdf</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>Dataset listing (accident stats, motor vehicle data)</t>
-        </is>
-      </c>
-      <c r="E120" s="6" t="inlineStr">
-        <is>
-          <t>Partial / Unconfirmed</t>
+          <t>Full judgment: nationwide interim road-safety directions, District Highway Safety Task Forces, blackspot rectification</t>
+        </is>
+      </c>
+      <c r="E120" s="8" t="inlineStr">
+        <is>
+          <t>Search-result only</t>
         </is>
       </c>
       <c r="F120" s="4" t="inlineStr">
         <is>
-          <t>Direct fetch returned HTTP 403 (blocks scrapers) - check manually</t>
+          <t>Hosted on Supreme Court's own official API domain - very high-confidence primary legal source</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>MoSPI - Statistical Year Book Ch.38 (Accident Statistics)</t>
+          <t>data.gov.in - Road Accidents dataset group</t>
         </is>
       </c>
       <c r="B121" s="18" t="inlineStr">
@@ -4359,25 +4363,29 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>https://mospi.gov.in/sites/default/files/Statistical_year_book_india_chapters/ch38.pdf</t>
+          <t>https://www.data.gov.in/dataset-group-name/Road%20Accidents</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>Statistical yearbook chapter (PDF)</t>
-        </is>
-      </c>
-      <c r="E121" s="8" t="inlineStr">
-        <is>
-          <t>Search-result only</t>
-        </is>
-      </c>
-      <c r="F121" s="4" t="inlineStr"/>
+          <t>Dataset listing (accident stats, motor vehicle data)</t>
+        </is>
+      </c>
+      <c r="E121" s="6" t="inlineStr">
+        <is>
+          <t>Partial / Unconfirmed</t>
+        </is>
+      </c>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
+          <t>Direct fetch returned HTTP 403 (blocks scrapers) - check manually</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>PIB - Road safety press releases (MoRTH-tagged)</t>
+          <t>MoSPI - Statistical Year Book Ch.38 (Accident Statistics)</t>
         </is>
       </c>
       <c r="B122" s="18" t="inlineStr">
@@ -4387,12 +4395,12 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in</t>
+          <t>https://mospi.gov.in/sites/default/files/Statistical_year_book_india_chapters/ch38.pdf</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>Press releases on rule changes, campaigns (e.g. Sadak Suraksha Abhiyaan, draft CMVR amendments)</t>
+          <t>Statistical yearbook chapter (PDF)</t>
         </is>
       </c>
       <c r="E122" s="8" t="inlineStr">
@@ -4400,31 +4408,27 @@
           <t>Search-result only</t>
         </is>
       </c>
-      <c r="F122" s="4" t="inlineStr">
-        <is>
-          <t>Ongoing 'what changed' feed, not a static repository - search filtered to MoRTH tag</t>
-        </is>
-      </c>
+      <c r="F122" s="4" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>CBIC/GST Council - GST rate notifications on motor vehicles</t>
-        </is>
-      </c>
-      <c r="B123" s="19" t="inlineStr">
-        <is>
-          <t>Tangential (low priority)</t>
+          <t>PIB - Road safety press releases (MoRTH-tagged)</t>
+        </is>
+      </c>
+      <c r="B123" s="18" t="inlineStr">
+        <is>
+          <t>Research/Data/Statistics</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>https://cbic-gst.gov.in/gst-goods-services-rates.html | https://www.gstcouncil.gov.in/cgst-rate-notification</t>
+          <t>https://www.pib.gov.in</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>Vehicle taxation notification PDFs</t>
+          <t>Press releases on rule changes, campaigns (e.g. Sadak Suraksha Abhiyaan, draft CMVR amendments)</t>
         </is>
       </c>
       <c r="E123" s="8" t="inlineStr">
@@ -4434,14 +4438,14 @@
       </c>
       <c r="F123" s="4" t="inlineStr">
         <is>
-          <t>Marginally 'traffic regulation' - vehicle taxation only</t>
+          <t>Ongoing 'what changed' feed, not a static repository - search filtered to MoRTH tag</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Ministry of Petroleum &amp; Natural Gas - Auto Fuel Policy / BS-VI</t>
+          <t>CBIC/GST Council - GST rate notifications on motor vehicles</t>
         </is>
       </c>
       <c r="B124" s="19" t="inlineStr">
@@ -4451,12 +4455,12 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>https://mopng.gov.in/en/refining/auto-fuel-policy</t>
+          <t>https://cbic-gst.gov.in/gst-goods-services-rates.html | https://www.gstcouncil.gov.in/cgst-rate-notification</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>Auto Fuel Vision &amp; Policy documents</t>
+          <t>Vehicle taxation notification PDFs</t>
         </is>
       </c>
       <c r="E124" s="8" t="inlineStr">
@@ -4466,14 +4470,14 @@
       </c>
       <c r="F124" s="4" t="inlineStr">
         <is>
-          <t>Fuel-quality policy, tangential to traffic rules</t>
+          <t>Marginally 'traffic regulation' - vehicle taxation only</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>MHA - Circulars &amp; National Advisories</t>
+          <t>Ministry of Petroleum &amp; Natural Gas - Auto Fuel Policy / BS-VI</t>
         </is>
       </c>
       <c r="B125" s="19" t="inlineStr">
@@ -4483,12 +4487,12 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>https://www.mha.gov.in/en/notifications/circular | https://www.mha.gov.in/en/documents/national-advisories</t>
+          <t>https://mopng.gov.in/en/refining/auto-fuel-policy</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>General home-affairs notification stream</t>
+          <t>Auto Fuel Vision &amp; Policy documents</t>
         </is>
       </c>
       <c r="E125" s="8" t="inlineStr">
@@ -4498,44 +4502,76 @@
       </c>
       <c r="F125" s="4" t="inlineStr">
         <is>
-          <t>Traffic/VIP-movement content appears only occasionally</t>
+          <t>Fuel-quality policy, tangential to traffic rules</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
+          <t>MHA - Circulars &amp; National Advisories</t>
+        </is>
+      </c>
+      <c r="B126" s="19" t="inlineStr">
+        <is>
+          <t>Tangential (low priority)</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mha.gov.in/en/notifications/circular | https://www.mha.gov.in/en/documents/national-advisories</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>General home-affairs notification stream</t>
+        </is>
+      </c>
+      <c r="E126" s="8" t="inlineStr">
+        <is>
+          <t>Search-result only</t>
+        </is>
+      </c>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>Traffic/VIP-movement content appears only occasionally</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
           <t>Election Commission of India - Election Laws (vehicle-use rules)</t>
         </is>
       </c>
-      <c r="B126" s="19" t="inlineStr">
+      <c r="B127" s="19" t="inlineStr">
         <is>
           <t>Tangential (low priority)</t>
         </is>
       </c>
-      <c r="C126" s="4" t="inlineStr">
+      <c r="C127" s="4" t="inlineStr">
         <is>
           <t>https://www.eci.gov.in/election-laws</t>
         </is>
       </c>
-      <c r="D126" s="4" t="inlineStr">
+      <c r="D127" s="4" t="inlineStr">
         <is>
           <t>Candidate/party vehicle-use rules on polling day</t>
         </is>
       </c>
-      <c r="E126" s="8" t="inlineStr">
+      <c r="E127" s="8" t="inlineStr">
         <is>
           <t>Search-result only</t>
         </is>
       </c>
-      <c r="F126" s="4" t="inlineStr">
+      <c r="F127" s="4" t="inlineStr">
         <is>
           <t>Real but narrow, single-purpose relevance</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F126"/>
+  <autoFilter ref="A1:F127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4652,7 +4688,7 @@
         </is>
       </c>
       <c r="B10" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
@@ -4692,7 +4728,7 @@
         </is>
       </c>
       <c r="B14" s="34" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16">
@@ -4752,7 +4788,7 @@
         </is>
       </c>
       <c r="B22" s="22" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23">

</xml_diff>